<commit_message>
dac and sinks and updated connections
</commit_message>
<xml_diff>
--- a/mes_north_sea/clean_data/nodes/nodes_2040.xlsx
+++ b/mes_north_sea/clean_data/nodes/nodes_2040.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maiant/PycharmProjects/Key-Infrastructure-North-Sea-CodeAndData/mes_north_sea/clean_data/nodes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A069BEBD-C8D5-1247-91B5-C89502974473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F570C56-6D06-1A44-BEF2-F34F45A49353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="160" yWindow="660" windowWidth="19260" windowHeight="15660" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes_used" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Nodes_all!$A$1:$E$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Nodes_used!$A$1:$B$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Nodes_used!$A$1:$B$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">storage_projects_all!$A$1:$P$48</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="223">
   <si>
     <t>Node</t>
   </si>
@@ -703,12 +703,6 @@
     <t>56.35, 4.67</t>
   </si>
   <si>
-    <t>DK_ST2</t>
-  </si>
-  <si>
-    <t>56.52, 9.98</t>
-  </si>
-  <si>
     <t>NO_ST1</t>
   </si>
   <si>
@@ -736,7 +730,7 @@
     <t>Trudvang &amp; Sleipner</t>
   </si>
   <si>
-    <t>No capacity announced for Net Zero Humber, placeholder at 500,000,000 like Greensand in NO</t>
+    <t>No capacity announced for Net Zero Humber, placeholder at 500,000,000 like Greensand in NO with the same injection rate</t>
   </si>
 </sst>
 </file>
@@ -1063,8 +1057,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C725760B-2CD8-914E-83CB-8DC400A3CB8A}" name="Table1" displayName="Table1" ref="A1:E72" totalsRowShown="0">
-  <autoFilter ref="A1:E72" xr:uid="{C725760B-2CD8-914E-83CB-8DC400A3CB8A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C725760B-2CD8-914E-83CB-8DC400A3CB8A}" name="Table1" displayName="Table1" ref="A1:E71" totalsRowShown="0">
+  <autoFilter ref="A1:E71" xr:uid="{C725760B-2CD8-914E-83CB-8DC400A3CB8A}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{D2D2E348-F8E9-9042-AEE1-9FE9D92AE0B3}" name="Node"/>
     <tableColumn id="2" xr3:uid="{CF5424B2-B747-8C43-A2F3-2A453817F318}" name="Type"/>
@@ -1079,8 +1073,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8198ECEC-84CC-8C4C-89D8-C0C7326FC773}" name="Table2" displayName="Table2" ref="A1:G17" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A1:G17" xr:uid="{8198ECEC-84CC-8C4C-89D8-C0C7326FC773}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8198ECEC-84CC-8C4C-89D8-C0C7326FC773}" name="Table2" displayName="Table2" ref="A1:G16" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:G16" xr:uid="{8198ECEC-84CC-8C4C-89D8-C0C7326FC773}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{D2330856-3D51-2447-BAD1-42FD070A7C83}" name="Project"/>
     <tableColumn id="2" xr3:uid="{E550573D-495D-FB4D-9952-E0A70DC9A0DD}" name="Country code"/>
@@ -1365,7 +1359,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K60"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.5" bestFit="1" customWidth="1"/>
@@ -2403,7 +2397,7 @@
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B58" t="s">
         <v>71</v>
@@ -2426,29 +2420,12 @@
         <v>71</v>
       </c>
       <c r="C59" t="s">
-        <v>72</v>
+        <v>98</v>
       </c>
       <c r="D59">
-        <v>9.98</v>
+        <v>1.9</v>
       </c>
       <c r="E59">
-        <v>56.52</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>215</v>
-      </c>
-      <c r="B60" t="s">
-        <v>71</v>
-      </c>
-      <c r="C60" t="s">
-        <v>98</v>
-      </c>
-      <c r="D60">
-        <v>1.9</v>
-      </c>
-      <c r="E60">
         <v>58.35</v>
       </c>
     </row>
@@ -3487,7 +3464,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDD3D8C9-E4BC-0046-BBBC-6939452B3EA0}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
@@ -3605,7 +3582,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B6" t="s">
         <v>61</v>
@@ -3625,19 +3602,19 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B7" t="s">
         <v>98</v>
       </c>
       <c r="C7" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D7" t="s">
         <v>211</v>
       </c>
       <c r="E7" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="F7" s="42">
         <v>720000000</v>
@@ -3648,179 +3625,176 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>107</v>
+        <v>208</v>
       </c>
       <c r="B8" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="C8" t="s">
-        <v>213</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>211</v>
-      </c>
-      <c r="E8" t="s">
-        <v>214</v>
+        <v>201</v>
       </c>
       <c r="F8" s="42">
-        <v>630000000</v>
+        <v>450000000</v>
       </c>
       <c r="G8">
-        <v>1712</v>
+        <v>3539</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>208</v>
+        <v>65</v>
       </c>
       <c r="B9" t="s">
         <v>61</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="D9" t="s">
         <v>201</v>
       </c>
       <c r="F9" s="42">
-        <v>450000000</v>
+        <v>126000000</v>
       </c>
       <c r="G9">
-        <v>3539</v>
+        <v>685</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>65</v>
+        <v>207</v>
       </c>
       <c r="B10" t="s">
-        <v>61</v>
+        <v>98</v>
       </c>
       <c r="C10" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="D10" t="s">
         <v>201</v>
       </c>
       <c r="F10" s="42">
-        <v>126000000</v>
+        <v>121000000</v>
       </c>
       <c r="G10">
-        <v>685</v>
+        <v>457</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>207</v>
+        <v>118</v>
       </c>
       <c r="B11" t="s">
-        <v>98</v>
+        <v>73</v>
       </c>
       <c r="C11" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="D11" t="s">
         <v>201</v>
       </c>
       <c r="F11" s="42">
-        <v>121000000</v>
+        <v>37000000</v>
       </c>
       <c r="G11">
-        <v>457</v>
+        <v>285</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>118</v>
+        <v>221</v>
       </c>
       <c r="B12" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>213</v>
       </c>
       <c r="D12" t="s">
-        <v>201</v>
+        <v>211</v>
+      </c>
+      <c r="E12" t="s">
+        <v>215</v>
       </c>
       <c r="F12" s="42">
-        <v>37000000</v>
+        <v>225000000</v>
       </c>
       <c r="G12">
-        <v>285</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>223</v>
+        <v>66</v>
       </c>
       <c r="B13" t="s">
-        <v>98</v>
+        <v>61</v>
       </c>
       <c r="C13" t="s">
-        <v>215</v>
+        <v>34</v>
       </c>
       <c r="D13" t="s">
-        <v>211</v>
-      </c>
-      <c r="E13" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="F13" s="42">
-        <v>225000000</v>
+        <v>300000000</v>
       </c>
       <c r="G13">
-        <v>1027</v>
+        <v>1712</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>66</v>
+        <v>206</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>98</v>
       </c>
       <c r="C14" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="D14" t="s">
         <v>201</v>
       </c>
       <c r="F14" s="42">
-        <v>300000000</v>
+        <v>215000000</v>
       </c>
       <c r="G14">
-        <v>1712</v>
+        <v>856</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>206</v>
+        <v>68</v>
       </c>
       <c r="B15" t="s">
-        <v>98</v>
+        <v>61</v>
       </c>
       <c r="C15" t="s">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="D15" t="s">
         <v>201</v>
       </c>
       <c r="F15" s="42">
-        <v>215000000</v>
+        <v>500000000</v>
       </c>
       <c r="G15">
-        <v>856</v>
+        <v>913</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>68</v>
+        <v>95</v>
       </c>
       <c r="B16" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="C16" t="s">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="D16" t="s">
         <v>201</v>
@@ -3832,39 +3806,19 @@
         <v>913</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>95</v>
-      </c>
-      <c r="B17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C17" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17" t="s">
-        <v>201</v>
-      </c>
-      <c r="F17" s="42">
-        <v>500000000</v>
-      </c>
-      <c r="G17">
-        <v>913</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18" s="43" t="s">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="43" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A20" s="43" t="s">
-        <v>224</v>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="43" t="s">
+        <v>222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>